<commit_message>
doc work Aug 10, 2026
</commit_message>
<xml_diff>
--- a/docs/project-management/time-log.xlsx
+++ b/docs/project-management/time-log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffkrystek/Jeff/yek_flashcard/docs/project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{194BCFE9-968D-6A4D-80E0-8A8B01702F74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E6EAA2C-F48B-744B-84FA-D84B674A408E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4780" yWindow="3780" windowWidth="27240" windowHeight="16180" xr2:uid="{0105DE84-9EB5-AE49-BB95-638DCEB5FCB9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="56">
   <si>
     <t>Date</t>
   </si>
@@ -198,6 +198,15 @@
   </si>
   <si>
     <t>general JSON formatting</t>
+  </si>
+  <si>
+    <t>decision log needs backfilled</t>
+  </si>
+  <si>
+    <t>KAN-59</t>
+  </si>
+  <si>
+    <t>general category and vocab overview</t>
   </si>
 </sst>
 </file>
@@ -939,10 +948,41 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
+      <c r="A20" s="1">
+        <v>46244</v>
+      </c>
+      <c r="B20">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
+      <c r="A21" s="1">
+        <v>46244</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
@@ -962,7 +1002,7 @@
       </c>
       <c r="B27">
         <f>SUM(B2:B24)</f>
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
updated daily log and time log
</commit_message>
<xml_diff>
--- a/docs/project-management/time-log.xlsx
+++ b/docs/project-management/time-log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffkrystek/Jeff/yek_flashcard/docs/project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E6EAA2C-F48B-744B-84FA-D84B674A408E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{878A60C7-8EBD-FA41-9ED4-321AFAD7B147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4780" yWindow="3780" windowWidth="27240" windowHeight="16180" xr2:uid="{0105DE84-9EB5-AE49-BB95-638DCEB5FCB9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="59">
   <si>
     <t>Date</t>
   </si>
@@ -207,6 +207,15 @@
   </si>
   <si>
     <t>general category and vocab overview</t>
+  </si>
+  <si>
+    <t>WBS, Risk Register, Roadmap</t>
+  </si>
+  <si>
+    <t>LLC research</t>
+  </si>
+  <si>
+    <t>KAN-22, KAN-15, KAN-14</t>
   </si>
 </sst>
 </file>
@@ -588,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98788C20-1FDB-4048-9CC4-A8CBA5635041}">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.33203125" customWidth="1"/>
@@ -985,10 +994,41 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
+      <c r="A22" s="1">
+        <v>46263</v>
+      </c>
+      <c r="B22">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E22" t="s">
+        <v>58</v>
+      </c>
+      <c r="F22" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
+      <c r="A23" s="1">
+        <v>46263</v>
+      </c>
+      <c r="B23">
+        <v>4</v>
+      </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
@@ -996,92 +1036,113 @@
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
     </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="1"/>
+    </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27">
-        <f>SUM(B2:B24)</f>
-        <v>47</v>
-      </c>
+      <c r="A27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="A30" s="1"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>16</v>
-      </c>
-      <c r="B31" t="s">
-        <v>17</v>
-      </c>
+      <c r="A31" s="1"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>18</v>
-      </c>
-      <c r="B32" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" t="s">
-        <v>21</v>
-      </c>
+      <c r="A32" s="1"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>22</v>
-      </c>
-      <c r="B34" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>24</v>
-      </c>
-      <c r="B35" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>11</v>
-      </c>
-      <c r="B36" t="s">
-        <v>26</v>
+        <v>39</v>
+      </c>
+      <c r="B34">
+        <f>SUM(B2:B31)</f>
+        <v>55</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>7</v>
-      </c>
-      <c r="B37" t="s">
-        <v>27</v>
+      <c r="A37" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B38" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
+        <v>18</v>
+      </c>
+      <c r="B39" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>22</v>
+      </c>
+      <c r="B41" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>24</v>
+      </c>
+      <c r="B42" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>11</v>
+      </c>
+      <c r="B43" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>28</v>
+      </c>
+      <c r="B45" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>30</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B46" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>